<commit_message>
fixing input and output excel sheets
</commit_message>
<xml_diff>
--- a/240718-I.xlsx
+++ b/240718-I.xlsx
@@ -1,17 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Lucas\TreadStone\label-maker\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D45D579-B123-4FA2-911A-2B8B0870ABB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22140" yWindow="3300" windowWidth="17475" windowHeight="8775"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Part #" sheetId="2" r:id="rId1"/>
     <sheet name="Property" sheetId="3" r:id="rId2"/>
     <sheet name="Summary" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,6 +29,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -30,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="46">
   <si>
     <t>Batch</t>
   </si>
@@ -113,9 +121,6 @@
     <t>Data</t>
   </si>
   <si>
-    <t>M40</t>
-  </si>
-  <si>
     <t>For the first shipment of an order, fill "Previous Shipment" column with 0's</t>
   </si>
   <si>
@@ -159,13 +164,25 @@
   </si>
   <si>
     <t>240718-I</t>
+  </si>
+  <si>
+    <t>M38</t>
+  </si>
+  <si>
+    <t>Pack #13</t>
+  </si>
+  <si>
+    <t>Pack #14</t>
+  </si>
+  <si>
+    <t>1110-038-2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -207,6 +224,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -216,7 +241,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -233,11 +258,56 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -255,7 +325,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -562,52 +656,132 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AI162"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AO162"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="9.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.85546875" customWidth="1"/>
+    <col min="2" max="2" width="9.7265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="18">
+        <v>26024</v>
+      </c>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
+      <c r="T1" s="16"/>
+      <c r="U1" s="16"/>
+      <c r="V1" s="16"/>
+      <c r="W1" s="16"/>
+      <c r="X1" s="16"/>
+      <c r="Y1" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z1" s="16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
+      <c r="S2" s="16"/>
+      <c r="T2" s="16"/>
+      <c r="U2" s="16"/>
+      <c r="V2" s="16"/>
+      <c r="W2" s="16"/>
+      <c r="X2" s="16"/>
+      <c r="Y2" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="16" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:35" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:35" ht="15.6" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+    <row r="3" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="19"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
+      <c r="S3" s="16"/>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="16"/>
+      <c r="W3" s="16"/>
+      <c r="X3" s="16"/>
+      <c r="Y3" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="19">
         <v>45491</v>
       </c>
     </row>
-    <row r="4" spans="1:35" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:41" x14ac:dyDescent="0.35">
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:35" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:41" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="1:35" s="8" customFormat="1" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:41" s="8" customFormat="1" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="8" t="s">
         <v>3</v>
       </c>
@@ -657,8 +831,17 @@
         <v>15</v>
       </c>
       <c r="AI6" s="9"/>
-    </row>
-    <row r="7" spans="1:35" s="8" customFormat="1" ht="15.6" x14ac:dyDescent="0.35">
+      <c r="AK6" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL6" s="16"/>
+      <c r="AM6" s="16"/>
+      <c r="AN6" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="AO6" s="16"/>
+    </row>
+    <row r="7" spans="1:41" s="8" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="10" t="s">
         <v>2</v>
       </c>
@@ -742,38 +925,31 @@
       <c r="AI7" s="11" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:35" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="1">
-        <v>95</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="1">
-        <v>22</v>
-      </c>
-      <c r="G8" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" s="1">
-        <v>23</v>
-      </c>
-      <c r="J8" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="K8" s="1">
-        <v>15</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="N8" s="1">
-        <v>21</v>
-      </c>
+      <c r="AK7" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="AL7" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="AM7" s="20"/>
+      <c r="AN7" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="AO7" s="21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="15"/>
+      <c r="B8" s="1"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="1"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="1"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
       <c r="S8" s="1"/>
@@ -789,39 +965,25 @@
       <c r="AG8" s="6"/>
       <c r="AH8" s="1"/>
       <c r="AI8" s="1"/>
-    </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="str">
-        <f>A8</f>
-        <v>M39</v>
-      </c>
-      <c r="B9" s="1">
-        <v>92</v>
-      </c>
-      <c r="D9" s="1" t="str">
-        <f>D8</f>
-        <v>M37</v>
-      </c>
-      <c r="E9" s="1">
-        <v>20</v>
-      </c>
-      <c r="G9" s="1" t="str">
-        <f>G8</f>
-        <v>M30</v>
-      </c>
-      <c r="H9" s="1">
-        <v>19</v>
-      </c>
-      <c r="J9" s="1" t="str">
-        <f>J8</f>
-        <v>M26</v>
-      </c>
-      <c r="K9" s="1">
-        <v>18</v>
-      </c>
+      <c r="AK8" s="17"/>
+      <c r="AL8" s="22"/>
+      <c r="AM8" s="16"/>
+      <c r="AN8" s="17"/>
+      <c r="AO8" s="18"/>
+    </row>
+    <row r="9" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
       <c r="S9" s="1"/>
       <c r="T9" s="1"/>
       <c r="V9" s="1"/>
@@ -835,36 +997,21 @@
       <c r="AG9" s="6"/>
       <c r="AH9" s="1"/>
       <c r="AI9" s="1"/>
-    </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="str">
-        <f t="shared" ref="A10:A23" si="0">A9</f>
-        <v>M39</v>
-      </c>
-      <c r="B10" s="1">
-        <v>98</v>
-      </c>
-      <c r="D10" s="1" t="str">
-        <f t="shared" ref="D10:D12" si="1">D9</f>
-        <v>M37</v>
-      </c>
-      <c r="E10" s="1">
-        <v>18</v>
-      </c>
-      <c r="G10" s="1" t="str">
-        <f t="shared" ref="G10:G13" si="2">G9</f>
-        <v>M30</v>
-      </c>
-      <c r="H10" s="1">
-        <v>25</v>
-      </c>
-      <c r="J10" s="1" t="str">
-        <f t="shared" ref="J10:J12" si="3">J9</f>
-        <v>M26</v>
-      </c>
-      <c r="K10" s="1">
-        <v>17</v>
-      </c>
+      <c r="AK9" s="17"/>
+      <c r="AL9" s="18"/>
+      <c r="AM9" s="16"/>
+      <c r="AN9" s="17"/>
+      <c r="AO9" s="18"/>
+    </row>
+    <row r="10" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
       <c r="P10" s="1"/>
@@ -882,36 +1029,21 @@
       <c r="AG10" s="6"/>
       <c r="AH10" s="1"/>
       <c r="AI10" s="1"/>
-    </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B11" s="1">
-        <v>87</v>
-      </c>
-      <c r="D11" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>M37</v>
-      </c>
-      <c r="E11" s="1">
-        <v>23</v>
-      </c>
-      <c r="G11" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>M30</v>
-      </c>
-      <c r="H11" s="1">
-        <v>22</v>
-      </c>
-      <c r="J11" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>M26</v>
-      </c>
-      <c r="K11" s="1">
-        <v>16</v>
-      </c>
+      <c r="AK10" s="17"/>
+      <c r="AL10" s="18"/>
+      <c r="AM10" s="16"/>
+      <c r="AN10" s="17"/>
+      <c r="AO10" s="18"/>
+    </row>
+    <row r="11" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="P11" s="1"/>
@@ -928,36 +1060,21 @@
       <c r="AG11" s="6"/>
       <c r="AH11" s="1"/>
       <c r="AI11" s="1"/>
-    </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B12" s="1">
-        <v>89</v>
-      </c>
-      <c r="D12" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>M37</v>
-      </c>
-      <c r="E12" s="1">
-        <v>21</v>
-      </c>
-      <c r="G12" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>M30</v>
-      </c>
-      <c r="H12" s="1">
-        <v>20</v>
-      </c>
-      <c r="J12" s="1" t="str">
-        <f t="shared" si="3"/>
-        <v>M26</v>
-      </c>
-      <c r="K12" s="1">
-        <v>21</v>
-      </c>
+      <c r="AK11" s="17"/>
+      <c r="AL11" s="18"/>
+      <c r="AM11" s="16"/>
+      <c r="AN11" s="17"/>
+      <c r="AO11" s="18"/>
+    </row>
+    <row r="12" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="P12" s="1"/>
@@ -975,22 +1092,17 @@
       <c r="AG12" s="6"/>
       <c r="AH12" s="1"/>
       <c r="AI12" s="1"/>
-    </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B13" s="1">
-        <v>94</v>
-      </c>
-      <c r="G13" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>M30</v>
-      </c>
-      <c r="H13" s="1">
-        <v>24</v>
-      </c>
+      <c r="AK12" s="17"/>
+      <c r="AL12" s="18"/>
+      <c r="AM12" s="16"/>
+      <c r="AN12" s="17"/>
+      <c r="AO12" s="18"/>
+    </row>
+    <row r="13" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
       <c r="P13" s="1"/>
@@ -1007,15 +1119,15 @@
       <c r="AG13" s="6"/>
       <c r="AH13" s="1"/>
       <c r="AI13" s="1"/>
-    </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B14" s="1">
-        <v>88</v>
-      </c>
+      <c r="AK13" s="17"/>
+      <c r="AL13" s="18"/>
+      <c r="AM13" s="16"/>
+      <c r="AN13" s="17"/>
+      <c r="AO13" s="18"/>
+    </row>
+    <row r="14" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="J14" s="1"/>
@@ -1037,15 +1149,15 @@
       <c r="AG14" s="6"/>
       <c r="AH14" s="1"/>
       <c r="AI14" s="1"/>
-    </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B15" s="1">
-        <v>93</v>
-      </c>
+      <c r="AK14" s="17"/>
+      <c r="AL14" s="18"/>
+      <c r="AM14" s="16"/>
+      <c r="AN14" s="17"/>
+      <c r="AO14" s="18"/>
+    </row>
+    <row r="15" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
       <c r="H15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
@@ -1065,15 +1177,15 @@
       <c r="AG15" s="6"/>
       <c r="AH15" s="1"/>
       <c r="AI15" s="1"/>
-    </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B16" s="1">
-        <v>99</v>
-      </c>
+      <c r="AK15" s="17"/>
+      <c r="AL15" s="18"/>
+      <c r="AM15" s="16"/>
+      <c r="AN15" s="17"/>
+      <c r="AO15" s="18"/>
+    </row>
+    <row r="16" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
       <c r="H16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
@@ -1094,15 +1206,15 @@
       <c r="AG16" s="6"/>
       <c r="AH16" s="1"/>
       <c r="AI16" s="1"/>
-    </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B17" s="1">
-        <v>100</v>
-      </c>
+      <c r="AK16" s="17"/>
+      <c r="AL16" s="18"/>
+      <c r="AM16" s="16"/>
+      <c r="AN16" s="17"/>
+      <c r="AO16" s="18"/>
+    </row>
+    <row r="17" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
       <c r="H17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
@@ -1122,15 +1234,15 @@
       <c r="AG17" s="6"/>
       <c r="AH17" s="1"/>
       <c r="AI17" s="1"/>
-    </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B18" s="1">
-        <v>97</v>
-      </c>
+      <c r="AK17" s="17"/>
+      <c r="AL17" s="18"/>
+      <c r="AM17" s="16"/>
+      <c r="AN17" s="17"/>
+      <c r="AO17" s="18"/>
+    </row>
+    <row r="18" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
       <c r="H18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -1151,15 +1263,15 @@
       <c r="AG18" s="6"/>
       <c r="AH18" s="1"/>
       <c r="AI18" s="1"/>
-    </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B19" s="1">
-        <v>86</v>
-      </c>
+      <c r="AK18" s="17"/>
+      <c r="AL18" s="18"/>
+      <c r="AM18" s="16"/>
+      <c r="AN18" s="17"/>
+      <c r="AO18" s="18"/>
+    </row>
+    <row r="19" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
       <c r="H19" s="1"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
@@ -1179,15 +1291,15 @@
       <c r="AG19" s="6"/>
       <c r="AH19" s="1"/>
       <c r="AI19" s="1"/>
-    </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B20" s="1">
-        <v>91</v>
-      </c>
+      <c r="AK19" s="17"/>
+      <c r="AL19" s="18"/>
+      <c r="AM19" s="16"/>
+      <c r="AN19" s="17"/>
+      <c r="AO19" s="18"/>
+    </row>
+    <row r="20" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
       <c r="H20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
@@ -1208,15 +1320,15 @@
       <c r="AG20" s="6"/>
       <c r="AH20" s="1"/>
       <c r="AI20" s="1"/>
-    </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B21" s="1">
-        <v>90</v>
-      </c>
+      <c r="AK20" s="17"/>
+      <c r="AL20" s="18"/>
+      <c r="AM20" s="16"/>
+      <c r="AN20" s="17"/>
+      <c r="AO20" s="18"/>
+    </row>
+    <row r="21" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="J21" s="1"/>
@@ -1237,15 +1349,15 @@
       <c r="AG21" s="6"/>
       <c r="AH21" s="1"/>
       <c r="AI21" s="1"/>
-    </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B22" s="1">
-        <v>85</v>
-      </c>
+      <c r="AK21" s="17"/>
+      <c r="AL21" s="18"/>
+      <c r="AM21" s="16"/>
+      <c r="AN21" s="17"/>
+      <c r="AO21" s="18"/>
+    </row>
+    <row r="22" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="J22" s="1"/>
@@ -1267,22 +1379,21 @@
       <c r="AG22" s="6"/>
       <c r="AH22" s="1"/>
       <c r="AI22" s="1"/>
-    </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>M39</v>
-      </c>
-      <c r="B23" s="1">
-        <v>96</v>
-      </c>
+      <c r="AK22" s="17"/>
+      <c r="AL22" s="18"/>
+      <c r="AM22" s="16"/>
+      <c r="AN22" s="17"/>
+      <c r="AO22" s="18"/>
+    </row>
+    <row r="23" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
-      <c r="P23" s="1"/>
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
       <c r="V23" s="1"/>
@@ -1296,8 +1407,13 @@
       <c r="AG23" s="6"/>
       <c r="AH23" s="1"/>
       <c r="AI23" s="1"/>
-    </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AK23" s="17"/>
+      <c r="AL23" s="18"/>
+      <c r="AM23" s="16"/>
+      <c r="AN23" s="17"/>
+      <c r="AO23" s="18"/>
+    </row>
+    <row r="24" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="G24" s="1"/>
@@ -1306,7 +1422,6 @@
       <c r="K24" s="1"/>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
-      <c r="P24" s="1"/>
       <c r="Q24" s="1"/>
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
@@ -1321,8 +1436,13 @@
       <c r="AG24" s="6"/>
       <c r="AH24" s="1"/>
       <c r="AI24" s="1"/>
-    </row>
-    <row r="25" spans="1:35" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="AK24" s="17"/>
+      <c r="AL24" s="18"/>
+      <c r="AM24" s="16"/>
+      <c r="AN24" s="17"/>
+      <c r="AO24" s="18"/>
+    </row>
+    <row r="25" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="D25" s="1"/>
@@ -1347,8 +1467,13 @@
       <c r="AG25" s="6"/>
       <c r="AH25" s="1"/>
       <c r="AI25" s="1"/>
-    </row>
-    <row r="26" spans="1:35" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="AK25" s="17"/>
+      <c r="AL25" s="18"/>
+      <c r="AM25" s="16"/>
+      <c r="AN25" s="17"/>
+      <c r="AO25" s="18"/>
+    </row>
+    <row r="26" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="D26" s="1"/>
@@ -1374,8 +1499,13 @@
       <c r="AG26" s="6"/>
       <c r="AH26" s="1"/>
       <c r="AI26" s="1"/>
-    </row>
-    <row r="27" spans="1:35" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="AK26" s="17"/>
+      <c r="AL26" s="18"/>
+      <c r="AM26" s="16"/>
+      <c r="AN26" s="17"/>
+      <c r="AO26" s="18"/>
+    </row>
+    <row r="27" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="D27" s="1"/>
@@ -1400,8 +1530,13 @@
       <c r="AG27" s="6"/>
       <c r="AH27" s="1"/>
       <c r="AI27" s="1"/>
-    </row>
-    <row r="28" spans="1:35" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="AK27" s="17"/>
+      <c r="AL27" s="18"/>
+      <c r="AM27" s="16"/>
+      <c r="AN27" s="17"/>
+      <c r="AO27" s="18"/>
+    </row>
+    <row r="28" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="D28" s="1"/>
@@ -1427,8 +1562,13 @@
       <c r="AG28" s="6"/>
       <c r="AH28" s="1"/>
       <c r="AI28" s="1"/>
-    </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AK28" s="17"/>
+      <c r="AL28" s="18"/>
+      <c r="AM28" s="16"/>
+      <c r="AN28" s="16"/>
+      <c r="AO28" s="16"/>
+    </row>
+    <row r="29" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="D29" s="1"/>
@@ -1453,8 +1593,13 @@
       <c r="AG29" s="6"/>
       <c r="AH29" s="1"/>
       <c r="AI29" s="1"/>
-    </row>
-    <row r="30" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AK29" s="17"/>
+      <c r="AL29" s="18"/>
+      <c r="AM29" s="16"/>
+      <c r="AN29" s="16"/>
+      <c r="AO29" s="16"/>
+    </row>
+    <row r="30" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="D30" s="1"/>
@@ -1480,8 +1625,13 @@
       <c r="AG30" s="6"/>
       <c r="AH30" s="1"/>
       <c r="AI30" s="1"/>
-    </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AK30" s="17"/>
+      <c r="AL30" s="18"/>
+      <c r="AM30" s="16"/>
+      <c r="AN30" s="16"/>
+      <c r="AO30" s="16"/>
+    </row>
+    <row r="31" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="D31" s="1"/>
@@ -1506,8 +1656,13 @@
       <c r="AG31" s="6"/>
       <c r="AH31" s="1"/>
       <c r="AI31" s="1"/>
-    </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AK31" s="17"/>
+      <c r="AL31" s="18"/>
+      <c r="AM31" s="16"/>
+      <c r="AN31" s="16"/>
+      <c r="AO31" s="16"/>
+    </row>
+    <row r="32" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="D32" s="1"/>
@@ -1534,7 +1689,7 @@
       <c r="AH32" s="1"/>
       <c r="AI32" s="1"/>
     </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="D33" s="1"/>
@@ -1560,7 +1715,7 @@
       <c r="AH33" s="1"/>
       <c r="AI33" s="1"/>
     </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="D34" s="1"/>
@@ -1587,554 +1742,431 @@
       <c r="AH34" s="1"/>
       <c r="AI34" s="1"/>
     </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B35" s="1">
-        <v>44</v>
-      </c>
-      <c r="D35" s="1">
-        <f t="shared" ref="D35:D36" si="4">D34</f>
-        <v>0</v>
-      </c>
-      <c r="E35" s="1">
-        <v>127</v>
-      </c>
-      <c r="G35" s="1">
-        <f t="shared" ref="G35:G36" si="5">G34</f>
-        <v>0</v>
-      </c>
-      <c r="H35" s="1">
-        <v>177</v>
-      </c>
-      <c r="J35" s="1">
-        <f t="shared" ref="J35:J36" si="6">J34</f>
-        <v>0</v>
-      </c>
-      <c r="K35" s="1">
-        <v>284</v>
-      </c>
-      <c r="M35" s="1">
-        <f t="shared" ref="M35:M36" si="7">M34</f>
-        <v>0</v>
-      </c>
-      <c r="N35" s="1">
-        <v>328</v>
-      </c>
-      <c r="P35" s="1">
-        <f t="shared" ref="P35:P36" si="8">P34</f>
-        <v>0</v>
-      </c>
-      <c r="Q35">
-        <v>357</v>
-      </c>
-      <c r="S35" s="1">
-        <f t="shared" ref="S35:S36" si="9">S34</f>
-        <v>0</v>
-      </c>
-      <c r="T35" s="1">
-        <v>386</v>
-      </c>
-      <c r="V35" s="1">
-        <f t="shared" ref="V35:V36" si="10">V34</f>
-        <v>0</v>
-      </c>
-      <c r="W35" s="1">
-        <v>427</v>
-      </c>
-      <c r="Y35" s="1">
-        <f t="shared" ref="Y35:Y36" si="11">Y34</f>
-        <v>0</v>
-      </c>
-      <c r="Z35" s="1">
-        <v>456</v>
-      </c>
-      <c r="AB35" s="1">
-        <f t="shared" ref="AB35:AB36" si="12">AB34</f>
-        <v>0</v>
-      </c>
-      <c r="AC35" s="1">
-        <v>485</v>
-      </c>
-      <c r="AE35" s="1">
-        <f t="shared" ref="AE35:AE36" si="13">AE34</f>
-        <v>0</v>
-      </c>
-      <c r="AF35" s="1">
-        <v>227</v>
-      </c>
+    <row r="35" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+      <c r="P35" s="1"/>
+      <c r="S35" s="1"/>
+      <c r="T35" s="1"/>
+      <c r="V35" s="1"/>
+      <c r="W35" s="1"/>
+      <c r="Y35" s="1"/>
+      <c r="Z35" s="1"/>
+      <c r="AB35" s="1"/>
+      <c r="AC35" s="1"/>
+      <c r="AE35" s="1"/>
+      <c r="AF35" s="1"/>
       <c r="AG35" s="4"/>
-      <c r="AH35" s="1">
-        <f t="shared" ref="AH35:AH36" si="14">AH34</f>
-        <v>0</v>
-      </c>
-      <c r="AI35" s="1">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B36" s="1">
-        <v>45</v>
-      </c>
-      <c r="D36" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E36" s="1">
-        <v>128</v>
-      </c>
-      <c r="G36" s="1">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="H36" s="1">
-        <v>178</v>
-      </c>
-      <c r="J36" s="1">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="K36" s="1">
-        <v>286</v>
-      </c>
-      <c r="M36" s="1">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="N36" s="1">
-        <v>329</v>
-      </c>
-      <c r="P36" s="1">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="Q36" s="1">
-        <v>358</v>
-      </c>
-      <c r="S36" s="1">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="T36" s="1">
-        <v>387</v>
-      </c>
-      <c r="V36" s="1">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="W36" s="1">
-        <v>428</v>
-      </c>
-      <c r="Y36" s="1">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="Z36" s="1">
-        <v>457</v>
-      </c>
-      <c r="AB36" s="1">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="AC36" s="1">
-        <v>486</v>
-      </c>
-      <c r="AE36" s="1">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="AF36" s="1">
-        <v>228</v>
-      </c>
+      <c r="AH35" s="1"/>
+      <c r="AI35" s="1"/>
+    </row>
+    <row r="36" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+      <c r="P36" s="1"/>
+      <c r="Q36" s="1"/>
+      <c r="S36" s="1"/>
+      <c r="T36" s="1"/>
+      <c r="V36" s="1"/>
+      <c r="W36" s="1"/>
+      <c r="Y36" s="1"/>
+      <c r="Z36" s="1"/>
+      <c r="AB36" s="1"/>
+      <c r="AC36" s="1"/>
+      <c r="AE36" s="1"/>
+      <c r="AF36" s="1"/>
       <c r="AG36" s="4"/>
-      <c r="AH36" s="1">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="AI36" s="1">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AH36" s="1"/>
+      <c r="AI36" s="1"/>
+    </row>
+    <row r="37" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A37" s="1"/>
     </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A38" s="1"/>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A39" s="1"/>
     </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
     </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A41" s="1"/>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A42" s="1"/>
     </row>
-    <row r="43" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A43" s="1"/>
     </row>
-    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A44" s="1"/>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A45" s="1"/>
     </row>
-    <row r="46" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A46" s="1"/>
     </row>
-    <row r="47" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A47" s="1"/>
     </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A48" s="1"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" s="1"/>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" s="1"/>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" s="1"/>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" s="1"/>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" s="1"/>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" s="1"/>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" s="1"/>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" s="1"/>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" s="1"/>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" s="1"/>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" s="1"/>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" s="1"/>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" s="1"/>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" s="1"/>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" s="1"/>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" s="1"/>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" s="1"/>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" s="1"/>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" s="1"/>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" s="1"/>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" s="1"/>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" s="1"/>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" s="1"/>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" s="1"/>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" s="1"/>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" s="1"/>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" s="1"/>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" s="1"/>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" s="1"/>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" s="1"/>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" s="1"/>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" s="1"/>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" s="1"/>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" s="1"/>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" s="1"/>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" s="1"/>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" s="1"/>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" s="1"/>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" s="1"/>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" s="1"/>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" s="1"/>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" s="1"/>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A91" s="1"/>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" s="1"/>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" s="1"/>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A94" s="1"/>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" s="1"/>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A96" s="1"/>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" s="1"/>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A98" s="1"/>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A99" s="1"/>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A100" s="1"/>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A101" s="1"/>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A102" s="1"/>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A103" s="1"/>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A104" s="1"/>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A105" s="1"/>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A106" s="1"/>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A107" s="1"/>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A108" s="1"/>
     </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A109" s="1"/>
     </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A110" s="1"/>
     </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A111" s="1"/>
     </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A112" s="1"/>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A113" s="1"/>
     </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A114" s="1"/>
     </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A115" s="1"/>
     </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A116" s="1"/>
     </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A117" s="1"/>
     </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A118" s="1"/>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A119" s="1"/>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A120" s="1"/>
     </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A121" s="1"/>
     </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A122" s="1"/>
     </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A123" s="1"/>
     </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A124" s="1"/>
     </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A125" s="1"/>
     </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A126" s="1"/>
     </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A127" s="1"/>
     </row>
-    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A128" s="1"/>
     </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A129" s="1"/>
     </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A130" s="1"/>
     </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A131" s="1"/>
     </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A132" s="1"/>
     </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A133" s="1"/>
     </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A134" s="1"/>
     </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A135" s="1"/>
     </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A136" s="1"/>
     </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A137" s="1"/>
     </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A138" s="1"/>
     </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A139" s="1"/>
     </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A140" s="1"/>
     </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A141" s="1"/>
     </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A142" s="1"/>
     </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A143" s="1"/>
     </row>
-    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A144" s="1"/>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A145" s="1"/>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A146" s="1"/>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A147" s="1"/>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A148" s="1"/>
     </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A149" s="1"/>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A150" s="1"/>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A151" s="1"/>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A152" s="1"/>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A153" s="1"/>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A154" s="1"/>
     </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A155" s="1"/>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A156" s="1"/>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A157" s="1"/>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A158" s="1"/>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A159" s="1"/>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A160" s="1"/>
     </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A161" s="1"/>
     </row>
-    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A162" s="1"/>
     </row>
   </sheetData>
@@ -2145,30 +2177,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="8.7109375" style="4"/>
+    <col min="2" max="2" width="8.7265625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>16</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="18.600000000000001" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="12" t="s">
         <v>2</v>
       </c>
@@ -2179,115 +2211,73 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="1">
-        <v>95</v>
-      </c>
-      <c r="C6" s="5">
-        <v>3.34</v>
-      </c>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="5"/>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="1">
-        <v>92</v>
-      </c>
-      <c r="C7" s="5">
-        <v>3.68</v>
-      </c>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="5"/>
       <c r="D7" s="3"/>
     </row>
-    <row r="8" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="1">
-        <v>22</v>
-      </c>
-      <c r="C8" s="5">
-        <v>4.8</v>
-      </c>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="5"/>
       <c r="D8" s="3"/>
     </row>
-    <row r="9" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="1">
-        <v>20</v>
-      </c>
-      <c r="C9" s="7">
-        <v>4.2699999999999996</v>
-      </c>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="7"/>
       <c r="D9" s="3"/>
     </row>
-    <row r="10" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="1">
-        <v>23</v>
-      </c>
-      <c r="C10" s="7">
-        <v>5.41</v>
-      </c>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="7"/>
       <c r="D10" s="3"/>
     </row>
-    <row r="11" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B11">
-        <v>15</v>
-      </c>
-      <c r="C11" s="5">
-        <v>5.05</v>
-      </c>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="1"/>
+      <c r="B11"/>
+      <c r="C11" s="5"/>
       <c r="D11" s="3"/>
     </row>
-    <row r="12" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12">
-        <v>21</v>
-      </c>
-      <c r="C12" s="5">
-        <v>3</v>
-      </c>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="1"/>
+      <c r="B12"/>
+      <c r="C12" s="5"/>
       <c r="D12" s="3"/>
     </row>
-    <row r="13" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13"/>
       <c r="C13" s="5"/>
       <c r="D13" s="3"/>
     </row>
-    <row r="14" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14"/>
       <c r="C14" s="5"/>
       <c r="D14" s="3"/>
     </row>
-    <row r="15" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="5"/>
       <c r="D15" s="3"/>
     </row>
-    <row r="16" spans="1:4" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="5"/>
       <c r="D16" s="3"/>
     </row>
-    <row r="17" spans="2:4" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B17" s="6"/>
       <c r="C17" s="5"/>
       <c r="D17" s="3"/>
@@ -2300,25 +2290,25 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:H22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="12.85546875" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="22.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" customWidth="1"/>
-    <col min="7" max="7" width="15.5703125" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" customWidth="1"/>
+    <col min="4" max="4" width="17.81640625" customWidth="1"/>
+    <col min="5" max="5" width="22.453125" customWidth="1"/>
+    <col min="6" max="6" width="14.453125" customWidth="1"/>
+    <col min="7" max="7" width="15.54296875" customWidth="1"/>
+    <col min="8" max="8" width="12.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="E2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.6" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>19</v>
       </c>
@@ -2344,212 +2334,161 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="14">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>4</v>
-      </c>
-      <c r="G4">
-        <f>F4+E4</f>
-        <v>4</v>
-      </c>
-      <c r="H4">
-        <f>D4-G4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="14">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>6</v>
-      </c>
-      <c r="G5">
-        <f t="shared" ref="G5:G8" si="0">F5+E5</f>
-        <v>6</v>
-      </c>
-      <c r="H5">
-        <f t="shared" ref="H5:H8" si="1">D5-G5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="14">
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="14">
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7">
-        <v>5</v>
-      </c>
-      <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7">
-        <v>5</v>
-      </c>
-      <c r="G7">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H7">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="14">
         <v>5</v>
       </c>
-      <c r="B8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
+      <c r="B8" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>42</v>
       </c>
       <c r="D8">
-        <v>16</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>16</v>
-      </c>
-      <c r="G8">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="H8">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="14">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+      <c r="B9" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="18">
+        <v>11</v>
+      </c>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="14">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="14">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="14">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="14">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="14">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="14">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="14">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="14">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="14">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="14">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="14">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="14">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="14.45" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" s="14">
         <v>0</v>
       </c>

</xml_diff>